<commit_message>
Seeded results: hourly pg_cron job in Supabase tops every daily game up to ~1000 plausible results a day (facade00- device ids), deletes seed rows after two days; build warns when the seed game list needs a migration
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Mannschaftssportarten_20x15.xlsx
+++ b/Mannschaftssportarten_20x15.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel.Keller\sportrankle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{659A5768-94AE-4A57-AABB-9C2FB79ACA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6942F287-7FE5-4795-9BAB-1C345FE4C32F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="28800" windowHeight="15225" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,7 +80,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="1">
+  <futureMetadata name="XLRICHVALUE" count="4">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -88,10 +88,40 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="1">
+  <valueMetadata count="4">
     <bk>
       <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -828,21 +858,75 @@
       </key>
     </keyFlags>
   </global>
+  <types>
+    <type name="_webimage">
+      <keyFlags>
+        <key name="WebImageIdentifier">
+          <flag name="ShowInCardView" value="0"/>
+        </key>
+      </keyFlags>
+    </type>
+  </types>
 </rvTypesInfo>
 </file>
 
+<file path=xl/richData/rdRichValueWebImage.xml><?xml version="1.0" encoding="utf-8"?>
+<webImagesSrd xmlns="http://schemas.microsoft.com/office/spreadsheetml/2020/richdatawebimage" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <webImageSrd>
+    <address r:id="rId1"/>
+    <blip r:id="rId2"/>
+  </webImageSrd>
+  <webImageSrd>
+    <address r:id="rId3"/>
+    <blip r:id="rId4"/>
+  </webImageSrd>
+  <webImageSrd>
+    <address r:id="rId5"/>
+    <blip r:id="rId6"/>
+  </webImageSrd>
+</webImagesSrd>
+</file>
+
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
   <rv s="0">
     <v>14</v>
+  </rv>
+  <rv s="1">
+    <v>0</v>
+    <v>1</v>
+    <v>0</v>
+    <v>0</v>
+    <v>Softball</v>
+  </rv>
+  <rv s="1">
+    <v>1</v>
+    <v>1</v>
+    <v>0</v>
+    <v>0</v>
+    <v>Unihockey</v>
+  </rv>
+  <rv s="1">
+    <v>2</v>
+    <v>1</v>
+    <v>0</v>
+    <v>0</v>
+    <v>Rollhockey</v>
   </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
   <s t="_error">
     <k n="errorType" t="i"/>
+  </s>
+  <s t="_webimage">
+    <k n="WebImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+    <k n="ComputedImage" t="b"/>
+    <k n="ImageSizing" t="i"/>
+    <k n="Text" t="s"/>
   </s>
 </rvStructures>
 </file>
@@ -1907,9 +1991,9 @@
       <c r="S14" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="T14" s="12" t="str">
-        <f ca="1">_xlfn.IMAGE(S14,"Softball",0)</f>
-        <v/>
+      <c r="T14" s="12" t="e" vm="2">
+        <f>_xlfn.IMAGE(S14,"Softball",0)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
@@ -2033,9 +2117,9 @@
       <c r="S16" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="T16" s="12" t="str">
-        <f ca="1">_xlfn.IMAGE(S16,"Unihockey",0)</f>
-        <v/>
+      <c r="T16" s="12" t="e" vm="3">
+        <f>_xlfn.IMAGE(S16,"Unihockey",0)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="1:20" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
@@ -2346,9 +2430,9 @@
       <c r="S21" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="T21" s="12" t="str">
-        <f ca="1">_xlfn.IMAGE(S21,"Rollhockey",0)</f>
-        <v/>
+      <c r="T21" s="12" t="e" vm="4">
+        <f>_xlfn.IMAGE(S21,"Rollhockey",0)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>